<commit_message>
Added regional markets to hydrogen.py. Called the demand_nodes analyses earlier in base.py. Other minor changes in LCI.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-distribution.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-distribution.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/premise/premise/data/additional_inventories/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390F1383-229A-014D-8BE8-2BAB8D47B4C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D743E9C5-A6FB-4E78-87C9-68687B612120}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="1600" windowWidth="25800" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="1596" windowWidth="25800" windowHeight="18036" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,8 +29,8 @@
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -853,7 +853,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -953,7 +953,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1232,15 +1232,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T364"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="44.5" customWidth="1"/>
+    <col min="1" max="1" width="44.44140625" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" customWidth="1"/>
     <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1248,7 +1249,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="15.6">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1256,7 +1257,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1264,7 +1265,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1272,7 +1273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1280,7 +1281,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1288,7 +1289,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1296,7 +1297,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1304,12 +1305,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" ht="15.6">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1338,7 +1339,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>155</v>
       </c>
@@ -1361,7 +1362,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" ht="15.6">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -1384,7 +1385,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" ht="15.6">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
@@ -1407,7 +1408,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" ht="15.6">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
@@ -1430,7 +1431,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="15.6">
       <c r="A16" s="2" t="s">
         <v>28</v>
       </c>
@@ -1453,7 +1454,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="15.6">
       <c r="A17" s="2" t="s">
         <v>30</v>
       </c>
@@ -1476,7 +1477,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="15.6">
       <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
@@ -1499,7 +1500,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="15.6">
       <c r="A19" s="2" t="s">
         <v>34</v>
       </c>
@@ -1522,7 +1523,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="15.6">
       <c r="A20" s="2" t="s">
         <v>36</v>
       </c>
@@ -1545,7 +1546,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="15.6">
       <c r="A21" s="2" t="s">
         <v>38</v>
       </c>
@@ -1568,7 +1569,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="15.6">
       <c r="A22" s="2" t="s">
         <v>40</v>
       </c>
@@ -1591,7 +1592,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="15.6">
       <c r="A23" s="2" t="s">
         <v>43</v>
       </c>
@@ -1614,7 +1615,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="15.6">
       <c r="A24" s="2" t="s">
         <v>45</v>
       </c>
@@ -1638,7 +1639,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="15.6">
       <c r="A25" s="2" t="s">
         <v>48</v>
       </c>
@@ -1662,7 +1663,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="15.6">
       <c r="A26" s="3" t="s">
         <v>111</v>
       </c>
@@ -1685,7 +1686,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="15.6">
       <c r="A28" s="1" t="s">
         <v>0</v>
       </c>
@@ -1693,7 +1694,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -1701,7 +1702,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>3</v>
       </c>
@@ -1709,7 +1710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -1717,7 +1718,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
         <v>6</v>
       </c>
@@ -1725,7 +1726,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16">
       <c r="A33" t="s">
         <v>7</v>
       </c>
@@ -1733,7 +1734,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -1741,12 +1742,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" ht="15.6">
       <c r="A35" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16">
       <c r="A36" t="s">
         <v>12</v>
       </c>
@@ -1775,7 +1776,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16">
       <c r="A37" t="s">
         <v>111</v>
       </c>
@@ -1798,7 +1799,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" ht="15.6">
       <c r="A38" s="2" t="s">
         <v>51</v>
       </c>
@@ -1821,7 +1822,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" ht="15.6">
       <c r="A39" s="2" t="s">
         <v>36</v>
       </c>
@@ -1844,7 +1845,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" ht="15.6">
       <c r="A40" s="2" t="s">
         <v>53</v>
       </c>
@@ -1867,7 +1868,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" ht="15.6">
       <c r="A41" s="2" t="s">
         <v>26</v>
       </c>
@@ -1890,7 +1891,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16">
       <c r="A42" t="s">
         <v>159</v>
       </c>
@@ -1913,7 +1914,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" ht="15.6">
       <c r="A43" s="2" t="s">
         <v>55</v>
       </c>
@@ -1936,7 +1937,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="44" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" ht="15.6">
       <c r="A44" s="2" t="s">
         <v>57</v>
       </c>
@@ -1959,7 +1960,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" ht="15.6">
       <c r="A45" s="2" t="s">
         <v>60</v>
       </c>
@@ -1982,7 +1983,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="46" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" ht="15.6">
       <c r="A46" s="2" t="s">
         <v>19</v>
       </c>
@@ -2005,7 +2006,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="48" spans="1:16" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" s="8" customFormat="1" ht="15.6">
       <c r="A48" s="7" t="s">
         <v>0</v>
       </c>
@@ -2019,7 +2020,7 @@
       <c r="O48" s="9"/>
       <c r="P48" s="9"/>
     </row>
-    <row r="49" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A49" s="8" t="s">
         <v>1</v>
       </c>
@@ -2033,7 +2034,7 @@
       <c r="O49" s="9"/>
       <c r="P49" s="9"/>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:20">
       <c r="A50" t="s">
         <v>161</v>
       </c>
@@ -2041,7 +2042,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="51" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A51" s="8" t="s">
         <v>3</v>
       </c>
@@ -2055,7 +2056,7 @@
       <c r="O51" s="9"/>
       <c r="P51" s="9"/>
     </row>
-    <row r="52" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A52" s="8" t="s">
         <v>4</v>
       </c>
@@ -2069,7 +2070,7 @@
       <c r="O52" s="9"/>
       <c r="P52" s="9"/>
     </row>
-    <row r="53" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A53" s="8" t="s">
         <v>6</v>
       </c>
@@ -2083,7 +2084,7 @@
       <c r="O53" s="9"/>
       <c r="P53" s="9"/>
     </row>
-    <row r="54" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A54" s="8" t="s">
         <v>9</v>
       </c>
@@ -2097,7 +2098,7 @@
       <c r="O54" s="9"/>
       <c r="P54" s="9"/>
     </row>
-    <row r="55" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A55" s="8" t="s">
         <v>7</v>
       </c>
@@ -2111,7 +2112,7 @@
       <c r="O55" s="9"/>
       <c r="P55" s="9"/>
     </row>
-    <row r="56" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A56" s="7" t="s">
         <v>11</v>
       </c>
@@ -2122,7 +2123,7 @@
       <c r="O56" s="9"/>
       <c r="P56" s="9"/>
     </row>
-    <row r="57" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A57" s="7" t="s">
         <v>12</v>
       </c>
@@ -2182,7 +2183,7 @@
       </c>
       <c r="T57" s="1"/>
     </row>
-    <row r="58" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A58" s="8" t="s">
         <v>160</v>
       </c>
@@ -2209,7 +2210,7 @@
       <c r="O58" s="9"/>
       <c r="P58" s="9"/>
     </row>
-    <row r="59" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A59" s="8" t="s">
         <v>175</v>
       </c>
@@ -2271,7 +2272,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="60" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A60" s="8" t="s">
         <v>176</v>
       </c>
@@ -2324,7 +2325,7 @@
       </c>
       <c r="T60"/>
     </row>
-    <row r="61" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A61" s="8" t="s">
         <v>177</v>
       </c>
@@ -2380,7 +2381,7 @@
       </c>
       <c r="T61"/>
     </row>
-    <row r="62" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A62" s="8" t="s">
         <v>179</v>
       </c>
@@ -2436,7 +2437,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="63" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A63" s="8" t="s">
         <v>182</v>
       </c>
@@ -2492,7 +2493,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="64" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A64" s="8" t="s">
         <v>183</v>
       </c>
@@ -2542,7 +2543,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="65" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A65" s="8" t="s">
         <v>186</v>
       </c>
@@ -2592,7 +2593,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="66" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A66" s="8" t="s">
         <v>187</v>
       </c>
@@ -2642,7 +2643,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="67" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A67" s="8" t="s">
         <v>188</v>
       </c>
@@ -2692,7 +2693,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="68" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A68" s="8" t="s">
         <v>189</v>
       </c>
@@ -2742,7 +2743,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="69" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A69" s="8" t="s">
         <v>191</v>
       </c>
@@ -2792,7 +2793,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="70" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A70" s="8" t="s">
         <v>193</v>
       </c>
@@ -2842,7 +2843,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="71" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A71" s="8" t="s">
         <v>193</v>
       </c>
@@ -2892,7 +2893,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="72" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="J72"/>
       <c r="K72" s="6"/>
       <c r="L72" s="6"/>
@@ -2903,7 +2904,7 @@
       <c r="Q72"/>
       <c r="R72"/>
     </row>
-    <row r="73" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A73" s="7" t="s">
         <v>0</v>
       </c>
@@ -2917,7 +2918,7 @@
       <c r="O73" s="9"/>
       <c r="P73" s="9"/>
     </row>
-    <row r="74" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:18" s="8" customFormat="1" ht="15">
       <c r="A74" s="8" t="s">
         <v>1</v>
       </c>
@@ -2931,7 +2932,7 @@
       <c r="O74" s="9"/>
       <c r="P74" s="9"/>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:18">
       <c r="A75" t="s">
         <v>161</v>
       </c>
@@ -2939,7 +2940,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="76" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:18" s="8" customFormat="1" ht="15">
       <c r="A76" s="8" t="s">
         <v>3</v>
       </c>
@@ -2953,7 +2954,7 @@
       <c r="O76" s="9"/>
       <c r="P76" s="9"/>
     </row>
-    <row r="77" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:18" s="8" customFormat="1" ht="15">
       <c r="A77" s="8" t="s">
         <v>4</v>
       </c>
@@ -2967,7 +2968,7 @@
       <c r="O77" s="9"/>
       <c r="P77" s="9"/>
     </row>
-    <row r="78" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:18" s="8" customFormat="1" ht="15">
       <c r="A78" s="8" t="s">
         <v>6</v>
       </c>
@@ -2981,7 +2982,7 @@
       <c r="O78" s="9"/>
       <c r="P78" s="9"/>
     </row>
-    <row r="79" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:18" s="8" customFormat="1" ht="15">
       <c r="A79" s="8" t="s">
         <v>9</v>
       </c>
@@ -2995,7 +2996,7 @@
       <c r="O79" s="9"/>
       <c r="P79" s="9"/>
     </row>
-    <row r="80" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:18" s="8" customFormat="1" ht="15">
       <c r="A80" s="8" t="s">
         <v>7</v>
       </c>
@@ -3009,7 +3010,7 @@
       <c r="O80" s="9"/>
       <c r="P80" s="9"/>
     </row>
-    <row r="81" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A81" s="7" t="s">
         <v>11</v>
       </c>
@@ -3020,7 +3021,7 @@
       <c r="O81" s="9"/>
       <c r="P81" s="9"/>
     </row>
-    <row r="82" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A82" s="7" t="s">
         <v>12</v>
       </c>
@@ -3080,7 +3081,7 @@
       </c>
       <c r="T82" s="1"/>
     </row>
-    <row r="83" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A83" s="8" t="str">
         <f>B73</f>
         <v>pipeline, hydrogen, high pressure transmission network</v>
@@ -3108,7 +3109,7 @@
       <c r="O83" s="9"/>
       <c r="P83" s="9"/>
     </row>
-    <row r="84" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A84" s="8" t="s">
         <v>197</v>
       </c>
@@ -3170,7 +3171,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="85" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A85" s="8" t="s">
         <v>198</v>
       </c>
@@ -3223,7 +3224,7 @@
       </c>
       <c r="T85"/>
     </row>
-    <row r="86" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A86" s="8" t="s">
         <v>199</v>
       </c>
@@ -3279,7 +3280,7 @@
       </c>
       <c r="T86"/>
     </row>
-    <row r="87" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A87" s="8" t="s">
         <v>179</v>
       </c>
@@ -3334,7 +3335,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="88" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A88" s="8" t="s">
         <v>182</v>
       </c>
@@ -3389,7 +3390,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="89" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A89" s="8" t="s">
         <v>183</v>
       </c>
@@ -3438,7 +3439,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="90" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A90" s="8" t="s">
         <v>186</v>
       </c>
@@ -3487,7 +3488,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="91" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A91" s="8" t="s">
         <v>187</v>
       </c>
@@ -3536,7 +3537,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="92" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A92" s="8" t="s">
         <v>188</v>
       </c>
@@ -3585,7 +3586,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="93" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A93" s="8" t="s">
         <v>189</v>
       </c>
@@ -3634,7 +3635,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="94" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A94" s="8" t="s">
         <v>191</v>
       </c>
@@ -3683,7 +3684,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="95" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A95" s="8" t="s">
         <v>193</v>
       </c>
@@ -3732,7 +3733,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="96" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A96" s="8" t="s">
         <v>193</v>
       </c>
@@ -3781,7 +3782,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="97" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="J97"/>
       <c r="K97" s="6"/>
       <c r="L97" s="6"/>
@@ -3792,7 +3793,7 @@
       <c r="Q97"/>
       <c r="R97"/>
     </row>
-    <row r="98" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A98" s="7" t="s">
         <v>0</v>
       </c>
@@ -3806,7 +3807,7 @@
       <c r="O98" s="9"/>
       <c r="P98" s="9"/>
     </row>
-    <row r="99" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A99" s="8" t="s">
         <v>1</v>
       </c>
@@ -3820,7 +3821,7 @@
       <c r="O99" s="9"/>
       <c r="P99" s="9"/>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:20">
       <c r="A100" t="s">
         <v>161</v>
       </c>
@@ -3828,7 +3829,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="101" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A101" s="8" t="s">
         <v>3</v>
       </c>
@@ -3842,7 +3843,7 @@
       <c r="O101" s="9"/>
       <c r="P101" s="9"/>
     </row>
-    <row r="102" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A102" s="8" t="s">
         <v>4</v>
       </c>
@@ -3856,7 +3857,7 @@
       <c r="O102" s="9"/>
       <c r="P102" s="9"/>
     </row>
-    <row r="103" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A103" s="8" t="s">
         <v>6</v>
       </c>
@@ -3870,7 +3871,7 @@
       <c r="O103" s="9"/>
       <c r="P103" s="9"/>
     </row>
-    <row r="104" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A104" s="8" t="s">
         <v>9</v>
       </c>
@@ -3884,7 +3885,7 @@
       <c r="O104" s="9"/>
       <c r="P104" s="9"/>
     </row>
-    <row r="105" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A105" s="8" t="s">
         <v>7</v>
       </c>
@@ -3898,7 +3899,7 @@
       <c r="O105" s="9"/>
       <c r="P105" s="9"/>
     </row>
-    <row r="106" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A106" s="7" t="s">
         <v>11</v>
       </c>
@@ -3909,7 +3910,7 @@
       <c r="O106" s="9"/>
       <c r="P106" s="9"/>
     </row>
-    <row r="107" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A107" s="7" t="s">
         <v>12</v>
       </c>
@@ -3969,7 +3970,7 @@
       </c>
       <c r="T107" s="1"/>
     </row>
-    <row r="108" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A108" s="8" t="str">
         <f>B98</f>
         <v>hydrogen distribution pipeline construction</v>
@@ -3996,7 +3997,7 @@
       <c r="O108" s="9"/>
       <c r="P108" s="9"/>
     </row>
-    <row r="109" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A109" s="13" t="s">
         <v>203</v>
       </c>
@@ -4061,7 +4062,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="110" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A110" s="13" t="s">
         <v>206</v>
       </c>
@@ -4116,7 +4117,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="111" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A111" s="13" t="s">
         <v>208</v>
       </c>
@@ -4171,7 +4172,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="112" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A112" s="13" t="s">
         <v>209</v>
       </c>
@@ -4226,7 +4227,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="113" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A113" s="8" t="s">
         <v>72</v>
       </c>
@@ -4281,7 +4282,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="114" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A114" s="13" t="s">
         <v>211</v>
       </c>
@@ -4336,7 +4337,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="115" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A115" s="13" t="s">
         <v>19</v>
       </c>
@@ -4391,7 +4392,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="116" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="J116"/>
       <c r="K116" s="6"/>
       <c r="L116" s="6"/>
@@ -4402,7 +4403,7 @@
       <c r="Q116"/>
       <c r="R116"/>
     </row>
-    <row r="117" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A117" s="7" t="s">
         <v>0</v>
       </c>
@@ -4416,7 +4417,7 @@
       <c r="O117" s="9"/>
       <c r="P117" s="9"/>
     </row>
-    <row r="118" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A118" s="8" t="s">
         <v>1</v>
       </c>
@@ -4430,7 +4431,7 @@
       <c r="O118" s="9"/>
       <c r="P118" s="9"/>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:20">
       <c r="A119" t="s">
         <v>161</v>
       </c>
@@ -4438,7 +4439,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="120" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A120" s="8" t="s">
         <v>3</v>
       </c>
@@ -4452,7 +4453,7 @@
       <c r="O120" s="9"/>
       <c r="P120" s="9"/>
     </row>
-    <row r="121" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A121" s="8" t="s">
         <v>4</v>
       </c>
@@ -4466,7 +4467,7 @@
       <c r="O121" s="9"/>
       <c r="P121" s="9"/>
     </row>
-    <row r="122" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A122" s="8" t="s">
         <v>6</v>
       </c>
@@ -4480,7 +4481,7 @@
       <c r="O122" s="9"/>
       <c r="P122" s="9"/>
     </row>
-    <row r="123" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A123" s="8" t="s">
         <v>9</v>
       </c>
@@ -4494,7 +4495,7 @@
       <c r="O123" s="9"/>
       <c r="P123" s="9"/>
     </row>
-    <row r="124" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A124" s="8" t="s">
         <v>7</v>
       </c>
@@ -4508,7 +4509,7 @@
       <c r="O124" s="9"/>
       <c r="P124" s="9"/>
     </row>
-    <row r="125" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A125" s="7" t="s">
         <v>11</v>
       </c>
@@ -4519,7 +4520,7 @@
       <c r="O125" s="9"/>
       <c r="P125" s="9"/>
     </row>
-    <row r="126" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A126" s="7" t="s">
         <v>12</v>
       </c>
@@ -4579,7 +4580,7 @@
       </c>
       <c r="T126" s="1"/>
     </row>
-    <row r="127" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A127" s="8" t="str">
         <f>B117</f>
         <v>hydrogen distribution pipeline installation</v>
@@ -4606,7 +4607,7 @@
       <c r="O127" s="9"/>
       <c r="P127" s="9"/>
     </row>
-    <row r="128" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A128" s="8" t="s">
         <v>69</v>
       </c>
@@ -4671,7 +4672,7 @@
         <v>0.79670949487272646</v>
       </c>
     </row>
-    <row r="129" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A129" s="8" t="s">
         <v>71</v>
       </c>
@@ -4726,7 +4727,7 @@
         <v>0.79670949487272646</v>
       </c>
     </row>
-    <row r="130" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A130" s="8" t="s">
         <v>213</v>
       </c>
@@ -4781,7 +4782,7 @@
         <v>0.71779376269979156</v>
       </c>
     </row>
-    <row r="131" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A131" s="8" t="s">
         <v>73</v>
       </c>
@@ -4836,7 +4837,7 @@
         <v>0.79670949487272646</v>
       </c>
     </row>
-    <row r="132" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="J132"/>
       <c r="K132" s="6"/>
       <c r="L132" s="6"/>
@@ -4847,7 +4848,7 @@
       <c r="Q132"/>
       <c r="R132"/>
     </row>
-    <row r="133" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A133" s="7" t="s">
         <v>0</v>
       </c>
@@ -4861,7 +4862,7 @@
       <c r="O133" s="9"/>
       <c r="P133" s="9"/>
     </row>
-    <row r="134" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A134" s="8" t="s">
         <v>1</v>
       </c>
@@ -4875,7 +4876,7 @@
       <c r="O134" s="9"/>
       <c r="P134" s="9"/>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:20">
       <c r="A135" t="s">
         <v>161</v>
       </c>
@@ -4883,7 +4884,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="136" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A136" s="8" t="s">
         <v>3</v>
       </c>
@@ -4897,7 +4898,7 @@
       <c r="O136" s="9"/>
       <c r="P136" s="9"/>
     </row>
-    <row r="137" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A137" s="8" t="s">
         <v>4</v>
       </c>
@@ -4911,7 +4912,7 @@
       <c r="O137" s="9"/>
       <c r="P137" s="9"/>
     </row>
-    <row r="138" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A138" s="8" t="s">
         <v>6</v>
       </c>
@@ -4925,7 +4926,7 @@
       <c r="O138" s="9"/>
       <c r="P138" s="9"/>
     </row>
-    <row r="139" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A139" s="8" t="s">
         <v>9</v>
       </c>
@@ -4939,7 +4940,7 @@
       <c r="O139" s="9"/>
       <c r="P139" s="9"/>
     </row>
-    <row r="140" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A140" s="8" t="s">
         <v>7</v>
       </c>
@@ -4953,7 +4954,7 @@
       <c r="O140" s="9"/>
       <c r="P140" s="9"/>
     </row>
-    <row r="141" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A141" s="7" t="s">
         <v>11</v>
       </c>
@@ -4964,7 +4965,7 @@
       <c r="O141" s="9"/>
       <c r="P141" s="9"/>
     </row>
-    <row r="142" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A142" s="7" t="s">
         <v>12</v>
       </c>
@@ -5024,7 +5025,7 @@
       </c>
       <c r="T142" s="1"/>
     </row>
-    <row r="143" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A143" s="8" t="str">
         <f>B133</f>
         <v>treatment of hydrogen distribution pipeline</v>
@@ -5052,7 +5053,7 @@
       <c r="O143" s="9"/>
       <c r="P143" s="9"/>
     </row>
-    <row r="144" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A144" s="8" t="s">
         <v>65</v>
       </c>
@@ -5120,7 +5121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A145" s="8" t="s">
         <v>216</v>
       </c>
@@ -5178,7 +5179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="K146" s="9"/>
       <c r="L146" s="9"/>
       <c r="M146" s="9"/>
@@ -5186,7 +5187,7 @@
       <c r="O146" s="9"/>
       <c r="P146" s="9"/>
     </row>
-    <row r="147" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A147" s="7" t="s">
         <v>0</v>
       </c>
@@ -5200,7 +5201,7 @@
       <c r="O147" s="9"/>
       <c r="P147" s="9"/>
     </row>
-    <row r="148" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A148" s="8" t="s">
         <v>1</v>
       </c>
@@ -5214,7 +5215,7 @@
       <c r="O148" s="9"/>
       <c r="P148" s="9"/>
     </row>
-    <row r="149" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:20">
       <c r="A149" t="s">
         <v>161</v>
       </c>
@@ -5222,7 +5223,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="150" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A150" s="8" t="s">
         <v>3</v>
       </c>
@@ -5236,7 +5237,7 @@
       <c r="O150" s="9"/>
       <c r="P150" s="9"/>
     </row>
-    <row r="151" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A151" s="8" t="s">
         <v>4</v>
       </c>
@@ -5250,7 +5251,7 @@
       <c r="O151" s="9"/>
       <c r="P151" s="9"/>
     </row>
-    <row r="152" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A152" s="8" t="s">
         <v>6</v>
       </c>
@@ -5264,7 +5265,7 @@
       <c r="O152" s="9"/>
       <c r="P152" s="9"/>
     </row>
-    <row r="153" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A153" s="8" t="s">
         <v>9</v>
       </c>
@@ -5278,7 +5279,7 @@
       <c r="O153" s="9"/>
       <c r="P153" s="9"/>
     </row>
-    <row r="154" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A154" s="8" t="s">
         <v>7</v>
       </c>
@@ -5292,7 +5293,7 @@
       <c r="O154" s="9"/>
       <c r="P154" s="9"/>
     </row>
-    <row r="155" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A155" s="7" t="s">
         <v>11</v>
       </c>
@@ -5303,7 +5304,7 @@
       <c r="O155" s="9"/>
       <c r="P155" s="9"/>
     </row>
-    <row r="156" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A156" s="7" t="s">
         <v>12</v>
       </c>
@@ -5363,7 +5364,7 @@
       </c>
       <c r="T156" s="1"/>
     </row>
-    <row r="157" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A157" s="8" t="str">
         <f>B147</f>
         <v>hydrogen transmission pipeline construction</v>
@@ -5390,7 +5391,7 @@
       <c r="O157" s="9"/>
       <c r="P157" s="9"/>
     </row>
-    <row r="158" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A158" s="13" t="s">
         <v>203</v>
       </c>
@@ -5455,7 +5456,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="159" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A159" s="13" t="s">
         <v>206</v>
       </c>
@@ -5510,7 +5511,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="160" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A160" s="13" t="s">
         <v>208</v>
       </c>
@@ -5565,7 +5566,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="161" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A161" s="13" t="s">
         <v>209</v>
       </c>
@@ -5620,7 +5621,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="162" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A162" s="8" t="s">
         <v>72</v>
       </c>
@@ -5675,7 +5676,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="163" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A163" s="13" t="s">
         <v>211</v>
       </c>
@@ -5730,7 +5731,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="164" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A164" s="13" t="s">
         <v>19</v>
       </c>
@@ -5785,7 +5786,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="165" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="J165"/>
       <c r="K165" s="6"/>
       <c r="L165" s="6"/>
@@ -5796,7 +5797,7 @@
       <c r="Q165"/>
       <c r="R165"/>
     </row>
-    <row r="166" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A166" s="7" t="s">
         <v>0</v>
       </c>
@@ -5810,7 +5811,7 @@
       <c r="O166" s="9"/>
       <c r="P166" s="9"/>
     </row>
-    <row r="167" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A167" s="8" t="s">
         <v>1</v>
       </c>
@@ -5824,7 +5825,7 @@
       <c r="O167" s="9"/>
       <c r="P167" s="9"/>
     </row>
-    <row r="168" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:20">
       <c r="A168" t="s">
         <v>161</v>
       </c>
@@ -5832,7 +5833,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="169" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A169" s="8" t="s">
         <v>3</v>
       </c>
@@ -5846,7 +5847,7 @@
       <c r="O169" s="9"/>
       <c r="P169" s="9"/>
     </row>
-    <row r="170" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A170" s="8" t="s">
         <v>4</v>
       </c>
@@ -5860,7 +5861,7 @@
       <c r="O170" s="9"/>
       <c r="P170" s="9"/>
     </row>
-    <row r="171" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A171" s="8" t="s">
         <v>6</v>
       </c>
@@ -5874,7 +5875,7 @@
       <c r="O171" s="9"/>
       <c r="P171" s="9"/>
     </row>
-    <row r="172" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A172" s="8" t="s">
         <v>9</v>
       </c>
@@ -5888,7 +5889,7 @@
       <c r="O172" s="9"/>
       <c r="P172" s="9"/>
     </row>
-    <row r="173" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A173" s="8" t="s">
         <v>7</v>
       </c>
@@ -5902,7 +5903,7 @@
       <c r="O173" s="9"/>
       <c r="P173" s="9"/>
     </row>
-    <row r="174" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A174" s="7" t="s">
         <v>11</v>
       </c>
@@ -5913,7 +5914,7 @@
       <c r="O174" s="9"/>
       <c r="P174" s="9"/>
     </row>
-    <row r="175" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A175" s="7" t="s">
         <v>12</v>
       </c>
@@ -5973,7 +5974,7 @@
       </c>
       <c r="T175" s="1"/>
     </row>
-    <row r="176" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A176" s="8" t="str">
         <f>B166</f>
         <v>hydrogen transmission pipeline installation</v>
@@ -6000,7 +6001,7 @@
       <c r="O176" s="9"/>
       <c r="P176" s="9"/>
     </row>
-    <row r="177" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A177" s="8" t="s">
         <v>69</v>
       </c>
@@ -6065,7 +6066,7 @@
         <v>0.79670949487272646</v>
       </c>
     </row>
-    <row r="178" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A178" s="8" t="s">
         <v>71</v>
       </c>
@@ -6120,7 +6121,7 @@
         <v>0.79670949487272646</v>
       </c>
     </row>
-    <row r="179" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A179" s="8" t="s">
         <v>213</v>
       </c>
@@ -6175,7 +6176,7 @@
         <v>0.71779376269979156</v>
       </c>
     </row>
-    <row r="180" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A180" s="8" t="s">
         <v>73</v>
       </c>
@@ -6230,7 +6231,7 @@
         <v>0.79670949487272646</v>
       </c>
     </row>
-    <row r="181" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="J181"/>
       <c r="K181" s="6"/>
       <c r="L181" s="6"/>
@@ -6241,7 +6242,7 @@
       <c r="Q181"/>
       <c r="R181"/>
     </row>
-    <row r="182" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A182" s="7" t="s">
         <v>0</v>
       </c>
@@ -6255,7 +6256,7 @@
       <c r="O182" s="9"/>
       <c r="P182" s="9"/>
     </row>
-    <row r="183" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A183" s="8" t="s">
         <v>1</v>
       </c>
@@ -6269,7 +6270,7 @@
       <c r="O183" s="9"/>
       <c r="P183" s="9"/>
     </row>
-    <row r="184" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:20">
       <c r="A184" t="s">
         <v>161</v>
       </c>
@@ -6277,7 +6278,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="185" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A185" s="8" t="s">
         <v>3</v>
       </c>
@@ -6291,7 +6292,7 @@
       <c r="O185" s="9"/>
       <c r="P185" s="9"/>
     </row>
-    <row r="186" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A186" s="8" t="s">
         <v>4</v>
       </c>
@@ -6305,7 +6306,7 @@
       <c r="O186" s="9"/>
       <c r="P186" s="9"/>
     </row>
-    <row r="187" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A187" s="8" t="s">
         <v>6</v>
       </c>
@@ -6319,7 +6320,7 @@
       <c r="O187" s="9"/>
       <c r="P187" s="9"/>
     </row>
-    <row r="188" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A188" s="8" t="s">
         <v>9</v>
       </c>
@@ -6333,7 +6334,7 @@
       <c r="O188" s="9"/>
       <c r="P188" s="9"/>
     </row>
-    <row r="189" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A189" s="8" t="s">
         <v>7</v>
       </c>
@@ -6347,7 +6348,7 @@
       <c r="O189" s="9"/>
       <c r="P189" s="9"/>
     </row>
-    <row r="190" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A190" s="7" t="s">
         <v>11</v>
       </c>
@@ -6358,7 +6359,7 @@
       <c r="O190" s="9"/>
       <c r="P190" s="9"/>
     </row>
-    <row r="191" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A191" s="7" t="s">
         <v>12</v>
       </c>
@@ -6418,7 +6419,7 @@
       </c>
       <c r="T191" s="1"/>
     </row>
-    <row r="192" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A192" s="8" t="str">
         <f>B182</f>
         <v>treatment of hydrogen transmission pipeline</v>
@@ -6446,7 +6447,7 @@
       <c r="O192" s="9"/>
       <c r="P192" s="9"/>
     </row>
-    <row r="193" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A193" s="8" t="s">
         <v>65</v>
       </c>
@@ -6514,7 +6515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A194" s="8" t="s">
         <v>216</v>
       </c>
@@ -6572,7 +6573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="K195" s="9"/>
       <c r="L195" s="9"/>
       <c r="M195" s="9"/>
@@ -6580,7 +6581,7 @@
       <c r="O195" s="9"/>
       <c r="P195" s="9"/>
     </row>
-    <row r="196" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A196" s="7" t="s">
         <v>0</v>
       </c>
@@ -6594,7 +6595,7 @@
       <c r="O196" s="9"/>
       <c r="P196" s="9"/>
     </row>
-    <row r="197" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A197" s="8" t="s">
         <v>1</v>
       </c>
@@ -6608,7 +6609,7 @@
       <c r="O197" s="9"/>
       <c r="P197" s="9"/>
     </row>
-    <row r="198" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:20">
       <c r="A198" t="s">
         <v>161</v>
       </c>
@@ -6616,7 +6617,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="199" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A199" s="8" t="s">
         <v>3</v>
       </c>
@@ -6630,7 +6631,7 @@
       <c r="O199" s="9"/>
       <c r="P199" s="9"/>
     </row>
-    <row r="200" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A200" s="8" t="s">
         <v>4</v>
       </c>
@@ -6644,7 +6645,7 @@
       <c r="O200" s="9"/>
       <c r="P200" s="9"/>
     </row>
-    <row r="201" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A201" s="8" t="s">
         <v>6</v>
       </c>
@@ -6658,7 +6659,7 @@
       <c r="O201" s="9"/>
       <c r="P201" s="9"/>
     </row>
-    <row r="202" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A202" s="8" t="s">
         <v>9</v>
       </c>
@@ -6672,7 +6673,7 @@
       <c r="O202" s="9"/>
       <c r="P202" s="9"/>
     </row>
-    <row r="203" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A203" s="8" t="s">
         <v>7</v>
       </c>
@@ -6686,7 +6687,7 @@
       <c r="O203" s="9"/>
       <c r="P203" s="9"/>
     </row>
-    <row r="204" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A204" s="7" t="s">
         <v>11</v>
       </c>
@@ -6697,7 +6698,7 @@
       <c r="O204" s="9"/>
       <c r="P204" s="9"/>
     </row>
-    <row r="205" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A205" s="7" t="s">
         <v>12</v>
       </c>
@@ -6757,7 +6758,7 @@
       </c>
       <c r="T205" s="1"/>
     </row>
-    <row r="206" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A206" s="8" t="s">
         <v>72</v>
       </c>
@@ -6783,7 +6784,7 @@
       <c r="O206" s="9"/>
       <c r="P206" s="9"/>
     </row>
-    <row r="207" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A207" s="8" t="s">
         <v>152</v>
       </c>
@@ -6848,7 +6849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A208" s="8" t="s">
         <v>148</v>
       </c>
@@ -6903,7 +6904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A209" s="8" t="s">
         <v>150</v>
       </c>
@@ -6958,7 +6959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A210" s="8" t="s">
         <v>77</v>
       </c>
@@ -7010,7 +7011,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="211" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A211" s="8" t="s">
         <v>256</v>
       </c>
@@ -7062,7 +7063,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="212" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A212" s="8" t="s">
         <v>80</v>
       </c>
@@ -7114,7 +7115,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="213" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A213" s="8" t="s">
         <v>82</v>
       </c>
@@ -7166,7 +7167,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="214" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A214" s="8" t="s">
         <v>84</v>
       </c>
@@ -7218,7 +7219,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="215" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A215" s="8" t="s">
         <v>220</v>
       </c>
@@ -7270,7 +7271,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="216" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A216" s="8" t="s">
         <v>89</v>
       </c>
@@ -7322,7 +7323,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="217" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A217" s="8" t="s">
         <v>91</v>
       </c>
@@ -7374,7 +7375,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="218" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A218" s="8" t="s">
         <v>221</v>
       </c>
@@ -7426,7 +7427,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="219" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A219" s="8" t="s">
         <v>257</v>
       </c>
@@ -7478,7 +7479,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="220" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A220" s="8" t="s">
         <v>94</v>
       </c>
@@ -7530,7 +7531,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="221" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A221" s="8" t="s">
         <v>156</v>
       </c>
@@ -7582,7 +7583,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="222" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A222" s="8" t="s">
         <v>57</v>
       </c>
@@ -7634,7 +7635,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="223" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A223" s="8" t="s">
         <v>96</v>
       </c>
@@ -7683,7 +7684,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="224" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A224" s="8" t="s">
         <v>222</v>
       </c>
@@ -7732,7 +7733,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="225" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A225" s="8" t="s">
         <v>99</v>
       </c>
@@ -7781,7 +7782,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="226" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A226" s="8" t="s">
         <v>223</v>
       </c>
@@ -7830,7 +7831,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="227" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A227" s="8" t="s">
         <v>101</v>
       </c>
@@ -7879,7 +7880,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="228" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A228" s="8" t="s">
         <v>102</v>
       </c>
@@ -7928,7 +7929,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="229" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A229" s="8" t="s">
         <v>103</v>
       </c>
@@ -7977,7 +7978,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="230" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A230" s="8" t="s">
         <v>224</v>
       </c>
@@ -8026,7 +8027,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="231" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A231" s="8" t="s">
         <v>225</v>
       </c>
@@ -8075,7 +8076,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="232" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A232" s="8" t="s">
         <v>104</v>
       </c>
@@ -8124,7 +8125,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="233" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A233" s="8" t="s">
         <v>226</v>
       </c>
@@ -8173,7 +8174,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="234" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A234" s="8" t="s">
         <v>227</v>
       </c>
@@ -8222,7 +8223,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="235" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A235" s="8" t="s">
         <v>227</v>
       </c>
@@ -8271,7 +8272,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="236" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A236" s="8" t="s">
         <v>228</v>
       </c>
@@ -8320,7 +8321,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="237" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A237" s="8" t="s">
         <v>228</v>
       </c>
@@ -8369,7 +8370,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="238" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A238" s="8" t="s">
         <v>229</v>
       </c>
@@ -8418,7 +8419,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="239" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A239" s="8" t="s">
         <v>105</v>
       </c>
@@ -8467,7 +8468,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="240" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A240" s="8" t="s">
         <v>106</v>
       </c>
@@ -8516,7 +8517,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="241" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A241" s="8" t="s">
         <v>107</v>
       </c>
@@ -8565,7 +8566,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="242" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A242" s="8" t="s">
         <v>108</v>
       </c>
@@ -8614,7 +8615,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="243" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A243" s="8" t="s">
         <v>230</v>
       </c>
@@ -8663,7 +8664,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="244" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A244" s="8" t="s">
         <v>230</v>
       </c>
@@ -8712,7 +8713,7 @@
         <v>0.93208283513358414</v>
       </c>
     </row>
-    <row r="245" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="K245" s="9"/>
       <c r="L245" s="9"/>
       <c r="M245" s="9"/>
@@ -8720,7 +8721,7 @@
       <c r="O245" s="9"/>
       <c r="P245" s="9"/>
     </row>
-    <row r="246" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A246" s="7" t="s">
         <v>0</v>
       </c>
@@ -8734,7 +8735,7 @@
       <c r="O246" s="9"/>
       <c r="P246" s="9"/>
     </row>
-    <row r="247" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A247" s="8" t="s">
         <v>1</v>
       </c>
@@ -8748,7 +8749,7 @@
       <c r="O247" s="9"/>
       <c r="P247" s="9"/>
     </row>
-    <row r="248" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:20">
       <c r="A248" t="s">
         <v>161</v>
       </c>
@@ -8756,7 +8757,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="249" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A249" s="8" t="s">
         <v>3</v>
       </c>
@@ -8770,7 +8771,7 @@
       <c r="O249" s="9"/>
       <c r="P249" s="9"/>
     </row>
-    <row r="250" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A250" s="8" t="s">
         <v>4</v>
       </c>
@@ -8784,7 +8785,7 @@
       <c r="O250" s="9"/>
       <c r="P250" s="9"/>
     </row>
-    <row r="251" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A251" s="8" t="s">
         <v>6</v>
       </c>
@@ -8798,7 +8799,7 @@
       <c r="O251" s="9"/>
       <c r="P251" s="9"/>
     </row>
-    <row r="252" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A252" s="8" t="s">
         <v>9</v>
       </c>
@@ -8812,7 +8813,7 @@
       <c r="O252" s="9"/>
       <c r="P252" s="9"/>
     </row>
-    <row r="253" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A253" s="8" t="s">
         <v>7</v>
       </c>
@@ -8826,7 +8827,7 @@
       <c r="O253" s="9"/>
       <c r="P253" s="9"/>
     </row>
-    <row r="254" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A254" s="7" t="s">
         <v>11</v>
       </c>
@@ -8837,7 +8838,7 @@
       <c r="O254" s="9"/>
       <c r="P254" s="9"/>
     </row>
-    <row r="255" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:20" s="8" customFormat="1" ht="15.6">
       <c r="A255" s="7" t="s">
         <v>12</v>
       </c>
@@ -8897,7 +8898,7 @@
       </c>
       <c r="T255" s="1"/>
     </row>
-    <row r="256" spans="1:20" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:20" s="8" customFormat="1" ht="15">
       <c r="A256" s="8" t="str">
         <f>B246</f>
         <v>compressor assembly for transmission hydrogen pipeline</v>
@@ -8927,7 +8928,7 @@
       <c r="O256" s="9"/>
       <c r="P256" s="9"/>
     </row>
-    <row r="257" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A257" s="13" t="s">
         <v>203</v>
       </c>
@@ -8989,7 +8990,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="258" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A258" s="8" t="s">
         <v>234</v>
       </c>
@@ -9041,7 +9042,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="259" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A259" s="8" t="s">
         <v>57</v>
       </c>
@@ -9093,7 +9094,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="260" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A260" s="8" t="s">
         <v>236</v>
       </c>
@@ -9145,7 +9146,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="261" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A261" s="8" t="s">
         <v>238</v>
       </c>
@@ -9197,7 +9198,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="262" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A262" s="8" t="s">
         <v>240</v>
       </c>
@@ -9249,7 +9250,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="263" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A263" s="8" t="s">
         <v>242</v>
       </c>
@@ -9301,7 +9302,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="264" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A264" s="8" t="s">
         <v>244</v>
       </c>
@@ -9353,7 +9354,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="265" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A265" s="8" t="s">
         <v>246</v>
       </c>
@@ -9405,7 +9406,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="266" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A266" s="8" t="s">
         <v>248</v>
       </c>
@@ -9457,7 +9458,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="267" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A267" s="8" t="s">
         <v>250</v>
       </c>
@@ -9509,7 +9510,7 @@
         <v>0.47095746419981693</v>
       </c>
     </row>
-    <row r="268" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A268" s="8" t="s">
         <v>73</v>
       </c>
@@ -9561,7 +9562,7 @@
         <v>0.58422518478336083</v>
       </c>
     </row>
-    <row r="269" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A269" s="8" t="s">
         <v>252</v>
       </c>
@@ -9616,7 +9617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="270" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A270" s="8" t="s">
         <v>254</v>
       </c>
@@ -9671,7 +9672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A271" s="8" t="s">
         <v>191</v>
       </c>
@@ -9720,7 +9721,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="272" spans="1:19" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:19" s="8" customFormat="1" ht="15.6">
       <c r="A272" s="8" t="s">
         <v>255</v>
       </c>
@@ -9769,7 +9770,7 @@
         <v>0.72314801614797197</v>
       </c>
     </row>
-    <row r="273" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A273" s="8" t="s">
         <v>193</v>
       </c>
@@ -9818,7 +9819,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="274" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:18" s="8" customFormat="1" ht="15.6">
       <c r="A274" s="8" t="s">
         <v>193</v>
       </c>
@@ -9867,7 +9868,7 @@
         <v>0.51215847306170115</v>
       </c>
     </row>
-    <row r="275" spans="1:18" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:18" s="8" customFormat="1" ht="15">
       <c r="B275" s="12"/>
       <c r="K275" s="9"/>
       <c r="L275" s="9"/>
@@ -9876,7 +9877,7 @@
       <c r="O275" s="9"/>
       <c r="P275" s="9"/>
     </row>
-    <row r="276" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:18" ht="15.6">
       <c r="A276" s="1" t="s">
         <v>0</v>
       </c>
@@ -9884,7 +9885,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="277" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:18">
       <c r="A277" t="s">
         <v>1</v>
       </c>
@@ -9892,7 +9893,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="278" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:18">
       <c r="A278" t="s">
         <v>3</v>
       </c>
@@ -9900,7 +9901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:18">
       <c r="A279" t="s">
         <v>4</v>
       </c>
@@ -9908,7 +9909,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="280" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:18">
       <c r="A280" t="s">
         <v>6</v>
       </c>
@@ -9916,7 +9917,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="281" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:18">
       <c r="A281" t="s">
         <v>9</v>
       </c>
@@ -9924,7 +9925,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="282" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:18">
       <c r="A282" t="s">
         <v>7</v>
       </c>
@@ -9932,12 +9933,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="283" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:18" ht="15.6">
       <c r="A283" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="284" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:18">
       <c r="A284" t="s">
         <v>12</v>
       </c>
@@ -9963,7 +9964,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="285" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:18" ht="15.6">
       <c r="A285" s="3" t="s">
         <v>113</v>
       </c>
@@ -9986,7 +9987,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="286" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:18">
       <c r="A286" t="s">
         <v>121</v>
       </c>
@@ -10009,7 +10010,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="287" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:18">
       <c r="A287" s="4" t="s">
         <v>118</v>
       </c>
@@ -10032,7 +10033,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="288" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:18">
       <c r="A288" t="s">
         <v>116</v>
       </c>
@@ -10055,7 +10056,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="289" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:8">
       <c r="A289" t="s">
         <v>125</v>
       </c>
@@ -10078,7 +10079,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="290" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:8">
       <c r="A290" t="s">
         <v>57</v>
       </c>
@@ -10101,7 +10102,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="292" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:8" ht="15.6">
       <c r="A292" s="1" t="s">
         <v>0</v>
       </c>
@@ -10109,7 +10110,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:8">
       <c r="A293" t="s">
         <v>1</v>
       </c>
@@ -10117,7 +10118,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="294" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:8">
       <c r="A294" t="s">
         <v>3</v>
       </c>
@@ -10125,7 +10126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="295" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:8">
       <c r="A295" t="s">
         <v>4</v>
       </c>
@@ -10133,7 +10134,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="296" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:8">
       <c r="A296" t="s">
         <v>6</v>
       </c>
@@ -10141,7 +10142,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="297" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:8">
       <c r="A297" t="s">
         <v>9</v>
       </c>
@@ -10149,7 +10150,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="298" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:8">
       <c r="A298" t="s">
         <v>7</v>
       </c>
@@ -10157,12 +10158,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="299" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:8" ht="15.6">
       <c r="A299" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="300" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:8">
       <c r="A300" t="s">
         <v>12</v>
       </c>
@@ -10188,7 +10189,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="301" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:8" ht="15.6">
       <c r="A301" s="3" t="s">
         <v>123</v>
       </c>
@@ -10211,7 +10212,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="302" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:8">
       <c r="A302" t="s">
         <v>121</v>
       </c>
@@ -10234,7 +10235,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="303" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:8">
       <c r="A303" s="4" t="s">
         <v>118</v>
       </c>
@@ -10257,7 +10258,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="304" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:8">
       <c r="A304" t="s">
         <v>116</v>
       </c>
@@ -10280,7 +10281,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="305" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:8">
       <c r="A305" t="s">
         <v>125</v>
       </c>
@@ -10303,7 +10304,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="306" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:8">
       <c r="A306" t="s">
         <v>57</v>
       </c>
@@ -10326,7 +10327,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="307" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:8">
       <c r="A307" t="s">
         <v>87</v>
       </c>
@@ -10350,7 +10351,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="309" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:8" ht="15.6">
       <c r="A309" s="1" t="s">
         <v>0</v>
       </c>
@@ -10358,7 +10359,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="310" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:8">
       <c r="A310" t="s">
         <v>1</v>
       </c>
@@ -10366,7 +10367,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="311" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:8">
       <c r="A311" t="s">
         <v>3</v>
       </c>
@@ -10374,7 +10375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="312" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:8">
       <c r="A312" t="s">
         <v>4</v>
       </c>
@@ -10382,7 +10383,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="313" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:8">
       <c r="A313" t="s">
         <v>6</v>
       </c>
@@ -10390,7 +10391,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="314" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:8">
       <c r="A314" t="s">
         <v>9</v>
       </c>
@@ -10398,7 +10399,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="315" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:8">
       <c r="A315" t="s">
         <v>7</v>
       </c>
@@ -10406,12 +10407,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="316" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:8" ht="15.6">
       <c r="A316" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="317" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:8">
       <c r="A317" t="s">
         <v>12</v>
       </c>
@@ -10437,7 +10438,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="318" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:8">
       <c r="A318" t="s">
         <v>125</v>
       </c>
@@ -10460,7 +10461,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="319" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:8">
       <c r="A319" t="s">
         <v>127</v>
       </c>
@@ -10483,7 +10484,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="320" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:8">
       <c r="A320" t="s">
         <v>129</v>
       </c>
@@ -10506,7 +10507,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="321" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:8">
       <c r="A321" t="s">
         <v>131</v>
       </c>
@@ -10529,7 +10530,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="322" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:8">
       <c r="A322" t="s">
         <v>134</v>
       </c>
@@ -10552,7 +10553,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="323" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:8">
       <c r="A323" t="s">
         <v>57</v>
       </c>
@@ -10575,7 +10576,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="324" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:8" ht="15.6">
       <c r="A324" s="3" t="s">
         <v>87</v>
       </c>
@@ -10598,7 +10599,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="325" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:8">
       <c r="A325" t="s">
         <v>156</v>
       </c>
@@ -10621,7 +10622,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="327" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:8" ht="15.6">
       <c r="A327" s="1" t="s">
         <v>0</v>
       </c>
@@ -10629,7 +10630,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="328" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:8">
       <c r="A328" t="s">
         <v>1</v>
       </c>
@@ -10637,7 +10638,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="329" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:8">
       <c r="A329" t="s">
         <v>3</v>
       </c>
@@ -10645,7 +10646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:8">
       <c r="A330" t="s">
         <v>4</v>
       </c>
@@ -10653,7 +10654,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="331" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:8">
       <c r="A331" t="s">
         <v>6</v>
       </c>
@@ -10661,7 +10662,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="332" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:8">
       <c r="A332" t="s">
         <v>9</v>
       </c>
@@ -10669,7 +10670,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="333" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:8">
       <c r="A333" t="s">
         <v>7</v>
       </c>
@@ -10677,12 +10678,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="334" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:8" ht="15.6">
       <c r="A334" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="335" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:8">
       <c r="A335" t="s">
         <v>12</v>
       </c>
@@ -10708,7 +10709,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="336" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:8">
       <c r="A336" t="s">
         <v>139</v>
       </c>
@@ -10731,7 +10732,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="337" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:8">
       <c r="A337" t="s">
         <v>57</v>
       </c>
@@ -10754,7 +10755,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="338" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:8">
       <c r="A338" t="s">
         <v>136</v>
       </c>
@@ -10777,7 +10778,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="340" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:8" ht="15.6">
       <c r="A340" s="1" t="s">
         <v>0</v>
       </c>
@@ -10785,7 +10786,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="341" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:8">
       <c r="A341" t="s">
         <v>1</v>
       </c>
@@ -10793,7 +10794,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="342" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:8">
       <c r="A342" t="s">
         <v>3</v>
       </c>
@@ -10801,7 +10802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="343" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:8">
       <c r="A343" t="s">
         <v>4</v>
       </c>
@@ -10809,7 +10810,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="344" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:8">
       <c r="A344" t="s">
         <v>6</v>
       </c>
@@ -10817,7 +10818,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="345" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:8">
       <c r="A345" t="s">
         <v>9</v>
       </c>
@@ -10825,7 +10826,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="346" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:8">
       <c r="A346" t="s">
         <v>7</v>
       </c>
@@ -10833,12 +10834,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="347" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:8" ht="15.6">
       <c r="A347" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="348" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:8">
       <c r="A348" t="s">
         <v>12</v>
       </c>
@@ -10864,7 +10865,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="349" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:8">
       <c r="A349" t="s">
         <v>140</v>
       </c>
@@ -10887,7 +10888,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="350" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:8">
       <c r="A350" t="s">
         <v>57</v>
       </c>
@@ -10910,7 +10911,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="351" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:8">
       <c r="A351" t="s">
         <v>139</v>
       </c>
@@ -10933,7 +10934,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="353" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:8" ht="15.6">
       <c r="A353" s="1" t="s">
         <v>0</v>
       </c>
@@ -10941,7 +10942,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="354" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:8">
       <c r="A354" t="s">
         <v>1</v>
       </c>
@@ -10949,7 +10950,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="355" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:8">
       <c r="A355" t="s">
         <v>3</v>
       </c>
@@ -10957,7 +10958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="356" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:8">
       <c r="A356" t="s">
         <v>4</v>
       </c>
@@ -10965,7 +10966,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="357" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:8">
       <c r="A357" t="s">
         <v>6</v>
       </c>
@@ -10973,7 +10974,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="358" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:8">
       <c r="A358" t="s">
         <v>9</v>
       </c>
@@ -10981,7 +10982,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="359" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:8">
       <c r="A359" t="s">
         <v>7</v>
       </c>
@@ -10989,12 +10990,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="360" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:8" ht="15.6">
       <c r="A360" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="361" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:8">
       <c r="A361" t="s">
         <v>12</v>
       </c>
@@ -11020,7 +11021,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="362" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:8">
       <c r="A362" t="s">
         <v>143</v>
       </c>
@@ -11043,7 +11044,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="363" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:8">
       <c r="A363" t="s">
         <v>57</v>
       </c>
@@ -11066,7 +11067,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="364" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:8">
       <c r="A364" t="s">
         <v>146</v>
       </c>

</xml_diff>